<commit_message>
update: upload latest CaseSize Format.xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Case Size.xlsx
+++ b/Case Size.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ee11846ce882123f/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="276" documentId="8_{B5CB9DC2-2DBC-48FC-8A4C-3FED4FBFDA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A254269-DFA7-44A7-96E3-8858676BCCEE}"/>
+  <xr:revisionPtr revIDLastSave="297" documentId="8_{B5CB9DC2-2DBC-48FC-8A4C-3FED4FBFDA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56518CD2-2572-42FA-B83D-418CBBC903D3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{94297B88-8998-40EB-8FA5-F929672964CF}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="99">
   <si>
     <t>Category</t>
   </si>
@@ -76,9 +76,6 @@
   </si>
   <si>
     <t>MASALA 15 GMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PREMIUM MASALA INCENSE HEXA </t>
   </si>
   <si>
     <t>24 Doz</t>
@@ -116,20 +113,6 @@
   <si>
     <r>
       <t>AROMA OIL</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color rgb="FF3D2020"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>CAR FRESHNER</t>
     </r>
     <r>
       <rPr>
@@ -409,12 +392,38 @@
   <si>
     <t>Candle Catalogue</t>
   </si>
+  <si>
+    <t>PREMIUM MASALA INCENSE (Hexa 15Stik)</t>
+  </si>
+  <si>
+    <r>
+      <t>CAR FRESHENER</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FF3D2020"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+  </si>
+  <si>
+    <t>ENERGY CLEANSING KIT</t>
+  </si>
+  <si>
+    <t>QATARI POWDER HEXA PACK</t>
+  </si>
+  <si>
+    <t>7 CHAKRA STONE</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="33" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -624,6 +633,12 @@
       <color rgb="FF1A0A0A"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="26">
@@ -9152,7 +9167,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{624BC790-9AE4-4E34-8AB5-C11F6DB95162}">
-  <dimension ref="A1:M80"/>
+  <dimension ref="A1:M81"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="41.453125" bestFit="1" customWidth="1"/>
@@ -9168,7 +9183,7 @@
   <sheetData>
     <row r="1" spans="1:10" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.6">
       <c r="A1" s="26" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C1" s="3"/>
       <c r="I1" s="13"/>
@@ -9204,11 +9219,11 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D3" s="3">
         <v>4</v>
@@ -9231,11 +9246,11 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D4" s="3">
         <v>8</v>
@@ -9258,11 +9273,11 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D5" s="3">
         <v>13</v>
@@ -9285,11 +9300,11 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3">
         <v>15.8</v>
@@ -9312,7 +9327,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="3" t="s">
@@ -9339,11 +9354,11 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D8" s="3">
         <v>9</v>
@@ -9366,11 +9381,11 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D9" s="3">
         <v>15</v>
@@ -9393,11 +9408,11 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D10" s="3">
         <v>16.5</v>
@@ -9420,7 +9435,7 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
-        <v>11</v>
+        <v>94</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="3" t="s">
@@ -9452,7 +9467,7 @@
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12" s="3">
         <v>10.3</v>
@@ -9476,11 +9491,11 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D13" s="3">
         <v>10.3</v>
@@ -9498,17 +9513,17 @@
         <v>45</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J13" s="5"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D14" s="3">
         <v>13.8</v>
@@ -9532,11 +9547,11 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D15" s="3">
         <v>13.8</v>
@@ -9560,11 +9575,11 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D16" s="3">
         <v>20.55</v>
@@ -9586,59 +9601,58 @@
       </c>
       <c r="J16" s="5"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
-        <v>21</v>
+        <v>98</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="3" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="D17" s="3">
+        <v>12</v>
+      </c>
+      <c r="E17" s="3">
+        <v>10</v>
+      </c>
+      <c r="F17" s="3">
+        <v>32.4</v>
+      </c>
+      <c r="G17" s="3">
         <v>15</v>
       </c>
-      <c r="E17" s="3">
-        <v>14.15</v>
-      </c>
-      <c r="F17" s="3">
-        <v>41</v>
-      </c>
-      <c r="G17" s="3">
-        <v>30</v>
-      </c>
       <c r="H17" s="3">
-        <v>45.5</v>
+        <v>32</v>
       </c>
       <c r="I17" s="15">
-        <v>5.5E-2</v>
-      </c>
-      <c r="J17" s="5"/>
+        <v>1.6E-2</v>
+      </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="7" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D18" s="3">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E18" s="3">
-        <v>6</v>
+        <v>14.15</v>
       </c>
       <c r="F18" s="3">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="G18" s="3">
-        <v>24.5</v>
+        <v>30</v>
       </c>
       <c r="H18" s="3">
-        <v>16</v>
+        <v>45.5</v>
       </c>
       <c r="I18" s="15">
-        <v>1.1368E-2</v>
+        <v>5.5E-2</v>
       </c>
       <c r="J18" s="5"/>
     </row>
@@ -9651,387 +9665,384 @@
         <v>19</v>
       </c>
       <c r="D19" s="3">
-        <v>9.6</v>
+        <v>7</v>
       </c>
       <c r="E19" s="3">
-        <v>8.85</v>
+        <v>6</v>
       </c>
       <c r="F19" s="3">
-        <v>31.5</v>
+        <v>29</v>
       </c>
       <c r="G19" s="3">
-        <v>27.5</v>
+        <v>24.5</v>
       </c>
       <c r="H19" s="3">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="I19" s="15">
-        <v>0.04</v>
-      </c>
-      <c r="J19" s="3"/>
+        <v>1.1368E-2</v>
+      </c>
+      <c r="J19" s="5"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A20" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="6"/>
+      <c r="A20" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="7"/>
       <c r="C20" s="3" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D20" s="3">
-        <v>6.5</v>
+        <v>9.6</v>
       </c>
       <c r="E20" s="3">
-        <v>5</v>
+        <v>8.85</v>
       </c>
       <c r="F20" s="3">
-        <v>33.5</v>
+        <v>31.5</v>
       </c>
       <c r="G20" s="3">
-        <v>29</v>
+        <v>27.5</v>
       </c>
       <c r="H20" s="3">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="I20" s="15">
-        <v>3.1088000000000001E-2</v>
+        <v>0.04</v>
       </c>
       <c r="J20" s="3"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
-        <v>26</v>
+        <v>95</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D21" s="3">
-        <v>8.3000000000000007</v>
+        <v>6.5</v>
       </c>
       <c r="E21" s="3">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="F21" s="3">
-        <v>38</v>
+        <v>33.5</v>
       </c>
       <c r="G21" s="3">
-        <v>33.5</v>
+        <v>29</v>
       </c>
       <c r="H21" s="3">
-        <v>28.5</v>
+        <v>32</v>
       </c>
       <c r="I21" s="15">
-        <v>3.5999999999999997E-2</v>
+        <v>3.1088000000000001E-2</v>
       </c>
       <c r="J21" s="3"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D22" s="3">
-        <v>10.4</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="E22" s="3">
-        <v>9.3000000000000007</v>
+        <v>7.5</v>
       </c>
       <c r="F22" s="3">
-        <v>34.5</v>
+        <v>38</v>
       </c>
       <c r="G22" s="3">
-        <v>26.5</v>
+        <v>33.5</v>
       </c>
       <c r="H22" s="3">
-        <v>48</v>
+        <v>28.5</v>
       </c>
       <c r="I22" s="15">
-        <v>4.3999999999999997E-2</v>
+        <v>3.5999999999999997E-2</v>
       </c>
       <c r="J22" s="3"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="3" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="D23" s="3">
-        <v>29.4</v>
+        <v>10.4</v>
       </c>
       <c r="E23" s="3">
-        <v>28</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="F23" s="3">
-        <v>45</v>
+        <v>34.5</v>
       </c>
       <c r="G23" s="3">
-        <v>41</v>
+        <v>26.5</v>
       </c>
       <c r="H23" s="3">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="I23" s="15">
-        <v>9.9629999999999996E-2</v>
+        <v>4.3999999999999997E-2</v>
       </c>
       <c r="J23" s="3"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="3" t="s">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D24" s="3">
-        <v>27</v>
+        <v>29.4</v>
       </c>
       <c r="E24" s="3">
-        <v>25.3</v>
+        <v>28</v>
       </c>
       <c r="F24" s="3">
-        <v>61.5</v>
+        <v>45</v>
       </c>
       <c r="G24" s="3">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="H24" s="3">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="I24" s="15">
-        <v>9.9015000000000006E-2</v>
+        <v>9.9629999999999996E-2</v>
       </c>
       <c r="J24" s="3"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="3" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="D25" s="3">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="E25" s="3">
-        <v>19</v>
+        <v>25.3</v>
       </c>
       <c r="F25" s="3">
-        <v>42.5</v>
+        <v>61.5</v>
       </c>
       <c r="G25" s="3">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="H25" s="3">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="I25" s="15">
-        <v>6.6640000000000005E-2</v>
+        <v>9.9015000000000006E-2</v>
       </c>
       <c r="J25" s="3"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="3" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="D26" s="3">
-        <v>12.75</v>
+        <v>20</v>
       </c>
       <c r="E26" s="3">
-        <v>11.2</v>
+        <v>19</v>
       </c>
       <c r="F26" s="3">
-        <v>37.5</v>
+        <v>42.5</v>
       </c>
       <c r="G26" s="3">
-        <v>28.2</v>
+        <v>32</v>
       </c>
       <c r="H26" s="3">
-        <v>34.799999999999997</v>
+        <v>49</v>
       </c>
       <c r="I26" s="15">
-        <v>3.6801E-2</v>
+        <v>6.6640000000000005E-2</v>
       </c>
       <c r="J26" s="3"/>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="3" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="D27" s="3">
-        <v>13.8</v>
+        <v>12.75</v>
       </c>
       <c r="E27" s="3">
-        <v>12.8</v>
+        <v>11.2</v>
       </c>
       <c r="F27" s="3">
-        <v>58.5</v>
+        <v>37.5</v>
       </c>
       <c r="G27" s="3">
-        <v>31</v>
+        <v>28.2</v>
       </c>
       <c r="H27" s="3">
-        <v>51.2</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="I27" s="15">
-        <v>9.2851200000000009E-2</v>
+        <v>3.6801E-2</v>
       </c>
       <c r="J27" s="3"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B28" s="6"/>
-      <c r="C28" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D28" s="9">
-        <v>13.5</v>
-      </c>
-      <c r="E28" s="9">
-        <v>12.4</v>
-      </c>
-      <c r="F28" s="9">
-        <v>47.5</v>
-      </c>
-      <c r="G28" s="9">
-        <v>44.3</v>
-      </c>
-      <c r="H28" s="9">
-        <v>32.5</v>
-      </c>
-      <c r="I28" s="14">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="J28" s="6"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="6"/>
+      <c r="C28" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="3">
+        <v>13.8</v>
+      </c>
+      <c r="E28" s="3">
+        <v>12.8</v>
+      </c>
+      <c r="F28" s="3">
+        <v>58.5</v>
+      </c>
+      <c r="G28" s="3">
+        <v>31</v>
+      </c>
+      <c r="H28" s="3">
+        <v>51.2</v>
+      </c>
+      <c r="I28" s="15">
+        <v>9.2851200000000009E-2</v>
+      </c>
+      <c r="J28" s="3"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="9" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="D29" s="9">
-        <v>15.3</v>
+        <v>13.5</v>
       </c>
       <c r="E29" s="9">
-        <v>13.95</v>
-      </c>
-      <c r="F29" s="9"/>
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
-      <c r="I29" s="14"/>
+        <v>12.4</v>
+      </c>
+      <c r="F29" s="9">
+        <v>47.5</v>
+      </c>
+      <c r="G29" s="9">
+        <v>44.3</v>
+      </c>
+      <c r="H29" s="9">
+        <v>32.5</v>
+      </c>
+      <c r="I29" s="14">
+        <v>7.0000000000000007E-2</v>
+      </c>
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
       <c r="L29" s="6"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="9" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D30" s="9">
-        <v>11</v>
+        <v>15.3</v>
       </c>
       <c r="E30" s="9">
-        <v>10</v>
-      </c>
-      <c r="F30" s="9">
-        <v>41.5</v>
-      </c>
-      <c r="G30" s="9">
-        <v>27.5</v>
-      </c>
-      <c r="H30" s="9">
-        <v>21</v>
-      </c>
-      <c r="I30" s="14">
-        <v>2.3966250000000001E-2</v>
-      </c>
+        <v>13.95</v>
+      </c>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="14"/>
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
       <c r="L30" s="6"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A31" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B31" s="7"/>
-      <c r="C31" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D31" s="3">
-        <v>15</v>
-      </c>
-      <c r="E31" s="3">
-        <v>14</v>
-      </c>
-      <c r="F31" s="3">
-        <v>63</v>
-      </c>
-      <c r="G31" s="3">
-        <v>32</v>
-      </c>
-      <c r="H31" s="3">
-        <v>41</v>
-      </c>
-      <c r="I31" s="15">
-        <v>8.2655999999999993E-2</v>
-      </c>
-      <c r="J31" s="18"/>
-      <c r="K31" s="18"/>
-      <c r="L31" s="18"/>
-      <c r="M31" s="18"/>
+      <c r="A31" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D31" s="9">
+        <v>11</v>
+      </c>
+      <c r="E31" s="9">
+        <v>10</v>
+      </c>
+      <c r="F31" s="9">
+        <v>41.5</v>
+      </c>
+      <c r="G31" s="9">
+        <v>27.5</v>
+      </c>
+      <c r="H31" s="9">
+        <v>21</v>
+      </c>
+      <c r="I31" s="14">
+        <v>2.3966250000000001E-2</v>
+      </c>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="3" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="D32" s="3">
-        <v>10.5</v>
+        <v>15</v>
       </c>
       <c r="E32" s="3">
-        <v>9.6999999999999993</v>
+        <v>14</v>
       </c>
       <c r="F32" s="3">
-        <v>37.5</v>
+        <v>63</v>
       </c>
       <c r="G32" s="3">
-        <v>30.5</v>
+        <v>32</v>
       </c>
       <c r="H32" s="3">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="I32" s="15">
-        <v>5.2999999999999999E-2</v>
+        <v>8.2655999999999993E-2</v>
       </c>
       <c r="J32" s="18"/>
       <c r="K32" s="18"/>
@@ -10040,29 +10051,29 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="3" t="s">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="D33" s="3">
-        <v>10.72</v>
+        <v>10.5</v>
       </c>
       <c r="E33" s="3">
-        <v>9.7200000000000006</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="F33" s="3">
-        <v>28</v>
+        <v>37.5</v>
       </c>
       <c r="G33" s="3">
-        <v>28</v>
+        <v>30.5</v>
       </c>
       <c r="H33" s="3">
-        <v>34.5</v>
+        <v>46</v>
       </c>
       <c r="I33" s="15">
-        <v>2.7047999999999999E-2</v>
+        <v>5.2999999999999999E-2</v>
       </c>
       <c r="J33" s="18"/>
       <c r="K33" s="18"/>
@@ -10071,29 +10082,29 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="3" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="D34" s="3">
-        <v>13</v>
+        <v>10.72</v>
       </c>
       <c r="E34" s="3">
-        <v>11</v>
+        <v>9.7200000000000006</v>
       </c>
       <c r="F34" s="3">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G34" s="3">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H34" s="3">
-        <v>39</v>
+        <v>34.5</v>
       </c>
       <c r="I34" s="15">
-        <v>0.03</v>
+        <v>2.7047999999999999E-2</v>
       </c>
       <c r="J34" s="18"/>
       <c r="K34" s="18"/>
@@ -10102,29 +10113,29 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="7" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="3" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="D35" s="3">
-        <v>11.4</v>
+        <v>13</v>
       </c>
       <c r="E35" s="3">
         <v>11</v>
       </c>
       <c r="F35" s="3">
-        <v>37.5</v>
+        <v>35</v>
       </c>
       <c r="G35" s="3">
-        <v>28.2</v>
+        <v>22</v>
       </c>
       <c r="H35" s="3">
-        <v>34.799999999999997</v>
+        <v>39</v>
       </c>
       <c r="I35" s="15">
-        <v>3.6801E-2</v>
+        <v>0.03</v>
       </c>
       <c r="J35" s="18"/>
       <c r="K35" s="18"/>
@@ -10133,29 +10144,29 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" s="7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="3" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="D36" s="3">
-        <v>23</v>
+        <v>11.4</v>
       </c>
       <c r="E36" s="3">
-        <v>21.5</v>
+        <v>11</v>
       </c>
       <c r="F36" s="3">
-        <v>41.5</v>
+        <v>37.5</v>
       </c>
       <c r="G36" s="3">
-        <v>41.5</v>
+        <v>28.2</v>
       </c>
       <c r="H36" s="3">
-        <v>54.7</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="I36" s="15">
-        <v>9.4207075000000001E-2</v>
+        <v>3.6801E-2</v>
       </c>
       <c r="J36" s="18"/>
       <c r="K36" s="18"/>
@@ -10164,29 +10175,29 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" s="7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B37" s="7"/>
       <c r="C37" s="3" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="D37" s="3">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E37" s="3">
-        <v>23</v>
+        <v>21.5</v>
       </c>
       <c r="F37" s="3">
-        <v>51.5</v>
+        <v>41.5</v>
       </c>
       <c r="G37" s="3">
-        <v>33.5</v>
+        <v>41.5</v>
       </c>
       <c r="H37" s="3">
-        <v>60</v>
+        <v>54.7</v>
       </c>
       <c r="I37" s="15">
-        <v>0.104</v>
+        <v>9.4207075000000001E-2</v>
       </c>
       <c r="J37" s="18"/>
       <c r="K37" s="18"/>
@@ -10194,23 +10205,38 @@
       <c r="M37" s="18"/>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A38" s="18"/>
-      <c r="B38" s="18"/>
-      <c r="C38" s="18"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="18"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="18"/>
+      <c r="A38" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B38" s="7"/>
+      <c r="C38" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" s="3">
+        <v>24</v>
+      </c>
+      <c r="E38" s="3">
+        <v>23</v>
+      </c>
+      <c r="F38" s="3">
+        <v>51.5</v>
+      </c>
+      <c r="G38" s="3">
+        <v>33.5</v>
+      </c>
+      <c r="H38" s="3">
+        <v>60</v>
+      </c>
+      <c r="I38" s="15">
+        <v>0.104</v>
+      </c>
       <c r="J38" s="18"/>
       <c r="K38" s="18"/>
       <c r="L38" s="18"/>
       <c r="M38" s="18"/>
     </row>
-    <row r="39" spans="1:13" ht="23" x14ac:dyDescent="0.35">
-      <c r="A39" s="20" t="s">
-        <v>71</v>
-      </c>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A39" s="18"/>
       <c r="B39" s="18"/>
       <c r="C39" s="18"/>
       <c r="D39" s="18"/>
@@ -10223,268 +10249,255 @@
       <c r="L39" s="18"/>
       <c r="M39" s="18"/>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A40" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D40" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="E40" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="F40" s="17" t="s">
-        <v>4</v>
-      </c>
-      <c r="G40" s="17" t="s">
-        <v>5</v>
-      </c>
-      <c r="H40" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="I40" s="16" t="s">
-        <v>7</v>
-      </c>
+    <row r="40" spans="1:13" ht="23" x14ac:dyDescent="0.35">
+      <c r="A40" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
       <c r="J40" s="18"/>
       <c r="K40" s="18"/>
       <c r="L40" s="18"/>
       <c r="M40" s="18"/>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A41" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B41" s="6"/>
-      <c r="C41" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
-      <c r="F41" s="3">
-        <v>50.9</v>
-      </c>
-      <c r="G41" s="3">
-        <v>39.6</v>
-      </c>
-      <c r="H41" s="3">
-        <v>60</v>
-      </c>
-      <c r="I41" s="15">
-        <v>0.12093840000000002</v>
-      </c>
-      <c r="J41" s="6"/>
+      <c r="A41" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D41" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="E41" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="F41" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="G41" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H41" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="I41" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="J41" s="18"/>
+      <c r="K41" s="18"/>
+      <c r="L41" s="18"/>
+      <c r="M41" s="18"/>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D42" s="3">
-        <v>27</v>
-      </c>
-      <c r="E42" s="3">
-        <v>24</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
       <c r="F42" s="3">
-        <v>55</v>
+        <v>50.9</v>
       </c>
       <c r="G42" s="3">
-        <v>33</v>
+        <v>39.6</v>
       </c>
       <c r="H42" s="3">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="I42" s="15">
-        <v>0.12705</v>
+        <v>0.12093840000000002</v>
       </c>
       <c r="J42" s="6"/>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="9" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="D43" s="3">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E43" s="3">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F43" s="3">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G43" s="3">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="H43" s="3">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="I43" s="15">
-        <v>0.11015999999999999</v>
+        <v>0.12705</v>
       </c>
       <c r="J43" s="6"/>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" s="6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B44" s="6"/>
-      <c r="C44" s="9"/>
+      <c r="C44" s="9" t="s">
+        <v>70</v>
+      </c>
       <c r="D44" s="3">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="E44" s="3">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="F44" s="3">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="G44" s="3">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H44" s="3">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="I44" s="15">
-        <v>7.0223999999999995E-2</v>
+        <v>0.11015999999999999</v>
       </c>
       <c r="J44" s="6"/>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" s="6" t="s">
-        <v>58</v>
+        <v>97</v>
       </c>
       <c r="B45" s="6"/>
-      <c r="C45" s="9" t="s">
-        <v>20</v>
-      </c>
+      <c r="C45" s="9"/>
       <c r="D45" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E45" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F45" s="3">
-        <v>46.5</v>
+        <v>38</v>
       </c>
       <c r="G45" s="3">
-        <v>36.5</v>
+        <v>56</v>
       </c>
       <c r="H45" s="3">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="I45" s="15">
-        <f>(F45*G45*H45)/1000000</f>
-        <v>9.3348749999999994E-2</v>
+        <v>7.0223999999999995E-2</v>
       </c>
       <c r="J45" s="6"/>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" s="6" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="9" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="D46" s="3">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="E46" s="3">
-        <v>9.3000000000000007</v>
+        <v>5</v>
       </c>
       <c r="F46" s="3">
-        <v>36</v>
+        <v>46.5</v>
       </c>
       <c r="G46" s="3">
-        <v>28</v>
+        <v>36.5</v>
       </c>
       <c r="H46" s="3">
-        <v>33.5</v>
+        <v>55</v>
       </c>
       <c r="I46" s="15">
         <f>(F46*G46*H46)/1000000</f>
-        <v>3.3767999999999999E-2</v>
+        <v>9.3348749999999994E-2</v>
       </c>
       <c r="J46" s="6"/>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" s="6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="9" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="D47" s="3">
-        <v>7</v>
+        <v>9.5</v>
       </c>
       <c r="E47" s="3">
-        <v>5</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="F47" s="3">
-        <v>46.5</v>
+        <v>36</v>
       </c>
       <c r="G47" s="3">
-        <v>36.5</v>
+        <v>28</v>
       </c>
       <c r="H47" s="3">
-        <v>55</v>
+        <v>33.5</v>
       </c>
       <c r="I47" s="15">
         <f>(F47*G47*H47)/1000000</f>
-        <v>9.3348749999999994E-2</v>
+        <v>3.3767999999999999E-2</v>
       </c>
       <c r="J47" s="6"/>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" s="6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="9" t="s">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="D48" s="3">
-        <v>10.3</v>
+        <v>7</v>
       </c>
       <c r="E48" s="3">
-        <v>9.6</v>
+        <v>5</v>
       </c>
       <c r="F48" s="3">
-        <v>49</v>
+        <v>46.5</v>
       </c>
       <c r="G48" s="3">
-        <v>27</v>
+        <v>36.5</v>
       </c>
       <c r="H48" s="3">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I48" s="15">
         <f>(F48*G48*H48)/1000000</f>
-        <v>5.9534999999999998E-2</v>
+        <v>9.3348749999999994E-2</v>
       </c>
       <c r="J48" s="6"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" s="6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D49" s="3">
         <v>10.3</v>
@@ -10502,128 +10515,129 @@
         <v>45</v>
       </c>
       <c r="I49" s="15">
-        <f t="shared" ref="I49" si="0">(F49*G49*H49)/1000000</f>
+        <f>(F49*G49*H49)/1000000</f>
         <v>5.9534999999999998E-2</v>
       </c>
       <c r="J49" s="6"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="6" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="9" t="s">
-        <v>73</v>
+        <v>11</v>
       </c>
       <c r="D50" s="3">
-        <v>10.72</v>
+        <v>10.3</v>
       </c>
       <c r="E50" s="3">
-        <v>9.7200000000000006</v>
+        <v>9.6</v>
       </c>
       <c r="F50" s="3">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="G50" s="3">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H50" s="3">
-        <v>34.5</v>
+        <v>45</v>
       </c>
       <c r="I50" s="15">
-        <v>2.7047999999999999E-2</v>
+        <f t="shared" ref="I50" si="0">(F50*G50*H50)/1000000</f>
+        <v>5.9534999999999998E-2</v>
       </c>
       <c r="J50" s="6"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" s="6" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D51" s="3">
-        <v>12.75</v>
+        <v>10.72</v>
       </c>
       <c r="E51" s="3">
-        <v>11.2</v>
+        <v>9.7200000000000006</v>
       </c>
       <c r="F51" s="3">
-        <v>37.5</v>
+        <v>28</v>
       </c>
       <c r="G51" s="3">
-        <v>28.2</v>
+        <v>28</v>
       </c>
       <c r="H51" s="3">
-        <v>34.799999999999997</v>
+        <v>34.5</v>
       </c>
       <c r="I51" s="15">
-        <v>3.6801E-2</v>
+        <v>2.7047999999999999E-2</v>
       </c>
       <c r="J51" s="6"/>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" s="6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B52" s="6"/>
-      <c r="C52" s="9"/>
+      <c r="C52" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="D52" s="3">
-        <v>16</v>
+        <v>12.75</v>
       </c>
       <c r="E52" s="3">
-        <v>15</v>
+        <v>11.2</v>
       </c>
       <c r="F52" s="3">
-        <v>22</v>
+        <v>37.5</v>
       </c>
       <c r="G52" s="3">
-        <v>7.8</v>
+        <v>28.2</v>
       </c>
       <c r="H52" s="3">
-        <v>21</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="I52" s="15">
-        <v>9.3348749999999994E-2</v>
+        <v>3.6801E-2</v>
       </c>
       <c r="J52" s="6"/>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" s="6" t="s">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="B53" s="6"/>
-      <c r="C53" s="9" t="s">
-        <v>37</v>
-      </c>
+      <c r="C53" s="9"/>
       <c r="D53" s="3">
-        <v>10.3</v>
+        <v>16</v>
       </c>
       <c r="E53" s="3">
-        <v>9.6</v>
+        <v>15</v>
       </c>
       <c r="F53" s="3">
-        <v>21.8</v>
+        <v>22</v>
       </c>
       <c r="G53" s="3">
-        <v>5.6</v>
+        <v>7.8</v>
       </c>
       <c r="H53" s="3">
-        <v>14.1</v>
+        <v>21</v>
       </c>
       <c r="I53" s="15">
-        <v>9.4E-2</v>
+        <v>9.3348749999999994E-2</v>
       </c>
       <c r="J53" s="6"/>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" s="6" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D54" s="3">
         <v>10.3</v>
@@ -10647,101 +10661,121 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="6" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="9" t="s">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="D55" s="3">
-        <v>15.6</v>
+        <v>10.3</v>
       </c>
       <c r="E55" s="3">
-        <v>14.6</v>
+        <v>9.6</v>
       </c>
       <c r="F55" s="3">
-        <v>54</v>
+        <v>21.8</v>
       </c>
       <c r="G55" s="3">
-        <v>30</v>
+        <v>5.6</v>
       </c>
       <c r="H55" s="3">
-        <v>44.5</v>
+        <v>14.1</v>
       </c>
       <c r="I55" s="15">
-        <f t="shared" ref="I55:I56" si="1">(F55*G55*H55)/1000000</f>
-        <v>7.2090000000000001E-2</v>
+        <v>9.4E-2</v>
       </c>
       <c r="J55" s="6"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="9" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="D56" s="3">
-        <v>20</v>
+        <v>15.6</v>
       </c>
       <c r="E56" s="3">
-        <v>19.2</v>
+        <v>14.6</v>
       </c>
       <c r="F56" s="3">
-        <v>48.5</v>
+        <v>54</v>
       </c>
       <c r="G56" s="3">
-        <v>40.5</v>
+        <v>30</v>
       </c>
       <c r="H56" s="3">
-        <v>42</v>
+        <v>44.5</v>
       </c>
       <c r="I56" s="15">
-        <f t="shared" si="1"/>
-        <v>8.2498500000000002E-2</v>
+        <f t="shared" ref="I56:I57" si="1">(F56*G56*H56)/1000000</f>
+        <v>7.2090000000000001E-2</v>
       </c>
       <c r="J56" s="6"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" s="6" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D57" s="3">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E57" s="3">
-        <v>28</v>
+        <v>19.2</v>
       </c>
       <c r="F57" s="3">
-        <f>12*4</f>
-        <v>48</v>
+        <v>48.5</v>
       </c>
       <c r="G57" s="3">
-        <f>25.5*2</f>
-        <v>51</v>
+        <v>40.5</v>
       </c>
       <c r="H57" s="3">
-        <f>2.5*18</f>
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I57" s="15">
-        <f>(F57*G57*H57)/1000000</f>
-        <v>0.11015999999999999</v>
+        <f t="shared" si="1"/>
+        <v>8.2498500000000002E-2</v>
       </c>
       <c r="J57" s="6"/>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="D58" s="3"/>
-      <c r="E58" s="3"/>
-      <c r="F58" s="3"/>
-      <c r="G58" s="3"/>
-      <c r="H58" s="3"/>
-      <c r="I58" s="15"/>
+      <c r="A58" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B58" s="6"/>
+      <c r="C58" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D58" s="3">
+        <v>30</v>
+      </c>
+      <c r="E58" s="3">
+        <v>28</v>
+      </c>
+      <c r="F58" s="3">
+        <f>12*4</f>
+        <v>48</v>
+      </c>
+      <c r="G58" s="3">
+        <f>25.5*2</f>
+        <v>51</v>
+      </c>
+      <c r="H58" s="3">
+        <f>2.5*18</f>
+        <v>45</v>
+      </c>
+      <c r="I58" s="15">
+        <f>(F58*G58*H58)/1000000</f>
+        <v>0.11015999999999999</v>
+      </c>
+      <c r="J58" s="6"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D59" s="3"/>
@@ -10751,368 +10785,377 @@
       <c r="H59" s="3"/>
       <c r="I59" s="15"/>
     </row>
-    <row r="60" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="A60" s="19" t="s">
-        <v>88</v>
-      </c>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="15"/>
     </row>
-    <row r="61" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="B61" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="C61" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="D61" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="E61" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="F61" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="G61" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="H61" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="I61" s="25" t="s">
-        <v>7</v>
+    <row r="61" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="A61" s="19" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="62" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D62" s="8">
+      <c r="A62" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B62" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C62" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="D62" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="E62" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="F62" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="G62" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="H62" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="I62" s="25" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A63" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D63" s="8">
         <v>9.6</v>
       </c>
-      <c r="E62" s="8">
+      <c r="E63" s="8">
         <v>8.8000000000000007</v>
       </c>
-      <c r="I62" s="13"/>
+      <c r="I63" s="13"/>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A63" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D63">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A64" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D64">
         <v>25</v>
       </c>
-      <c r="E63">
+      <c r="E64">
         <v>24</v>
       </c>
     </row>
-    <row r="64" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D64" s="8">
+    <row r="65" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A65" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65" s="8">
         <v>12.55</v>
       </c>
-      <c r="E64" s="8">
+      <c r="E65" s="8">
         <v>11.45</v>
       </c>
-      <c r="I64" s="13"/>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A65" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="D65">
-        <v>15.7</v>
-      </c>
-      <c r="E65">
-        <v>14.7</v>
-      </c>
+      <c r="I65" s="13"/>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" s="6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D66">
-        <v>15.2</v>
+        <v>15.7</v>
       </c>
       <c r="E66">
-        <v>14.2</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" s="6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="D67">
+        <v>15.2</v>
+      </c>
+      <c r="E67">
+        <v>14.2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A68" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D68">
         <v>13.2</v>
       </c>
-      <c r="E67">
+      <c r="E68">
         <v>12.5</v>
       </c>
     </row>
-    <row r="68" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D68">
+    <row r="69" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D69">
         <v>18.86</v>
       </c>
-      <c r="E68">
+      <c r="E69">
         <v>17.239999999999998</v>
       </c>
-      <c r="I68" s="13"/>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A69" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D69" s="8">
-        <v>17.600000000000001</v>
-      </c>
-      <c r="E69" s="8">
-        <v>16.600000000000001</v>
-      </c>
+      <c r="I69" s="13"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" s="6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D70">
-        <v>28.5</v>
-      </c>
-      <c r="E70">
-        <v>27</v>
+        <v>80</v>
+      </c>
+      <c r="D70" s="8">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="E70" s="8">
+        <v>16.600000000000001</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A71" s="6"/>
+      <c r="A71" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D71">
+        <v>28.5</v>
+      </c>
+      <c r="E71">
+        <v>27</v>
+      </c>
     </row>
-    <row r="72" spans="1:9" s="8" customFormat="1" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="A72" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="C72" s="3"/>
-      <c r="I72" s="13"/>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A72" s="6"/>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A73" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="B73" s="22" t="s">
-        <v>1</v>
-      </c>
-      <c r="C73" s="23" t="s">
-        <v>8</v>
-      </c>
-      <c r="D73" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="E73" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="F73" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="G73" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="H73" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="I73" s="25" t="s">
-        <v>7</v>
-      </c>
+    <row r="73" spans="1:9" s="8" customFormat="1" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="A73" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="C73" s="3"/>
+      <c r="I73" s="13"/>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A74" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C74" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D74">
-        <v>11.8</v>
-      </c>
-      <c r="E74">
-        <v>11.6</v>
-      </c>
-      <c r="F74">
-        <v>28.4</v>
-      </c>
-      <c r="G74">
-        <v>31.6</v>
-      </c>
-      <c r="H74">
-        <v>30</v>
-      </c>
-      <c r="I74" s="13">
-        <v>2.7E-2</v>
+      <c r="A74" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B74" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="C74" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="D74" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="E74" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="F74" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="G74" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="H74" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="I74" s="25" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" s="6" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="D75">
-        <v>12.75</v>
+        <v>11.8</v>
       </c>
       <c r="E75">
-        <v>11.2</v>
+        <v>11.6</v>
       </c>
       <c r="F75">
-        <v>37.5</v>
+        <v>28.4</v>
       </c>
       <c r="G75">
-        <v>28.2</v>
+        <v>31.6</v>
       </c>
       <c r="H75">
-        <v>34.799999999999997</v>
+        <v>30</v>
       </c>
       <c r="I75" s="13">
-        <v>3.6999999999999998E-2</v>
+        <v>2.7E-2</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A76" s="6" t="s">
-        <v>91</v>
+        <v>30</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>94</v>
+        <v>31</v>
       </c>
       <c r="D76">
-        <v>12</v>
+        <v>12.75</v>
       </c>
       <c r="E76">
-        <v>11.23</v>
+        <v>11.2</v>
       </c>
       <c r="F76">
-        <v>36</v>
+        <v>37.5</v>
       </c>
       <c r="G76">
-        <v>27</v>
+        <v>28.2</v>
       </c>
       <c r="H76">
-        <v>27</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="I76" s="13">
-        <v>2.6244E-2</v>
+        <v>3.6999999999999998E-2</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A77" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C77" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C77" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="D77">
-        <v>12.75</v>
+        <v>12</v>
       </c>
       <c r="E77">
-        <v>11.2</v>
+        <v>11.23</v>
       </c>
       <c r="F77">
-        <v>37.5</v>
+        <v>36</v>
       </c>
       <c r="G77">
-        <v>28.2</v>
+        <v>27</v>
       </c>
       <c r="H77">
-        <v>34.799999999999997</v>
+        <v>27</v>
       </c>
       <c r="I77" s="13">
-        <v>3.6999999999999998E-2</v>
+        <v>2.6244E-2</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A78" s="6" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="D78">
-        <v>11</v>
+        <v>12.75</v>
       </c>
       <c r="E78">
-        <v>13</v>
+        <v>11.2</v>
       </c>
       <c r="F78">
-        <v>35</v>
+        <v>37.5</v>
       </c>
       <c r="G78">
-        <v>22</v>
+        <v>28.2</v>
       </c>
       <c r="H78">
-        <v>39</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="I78" s="13">
-        <v>0.03</v>
+        <v>3.6999999999999998E-2</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" s="6" t="s">
-        <v>93</v>
+        <v>42</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="D79">
-        <v>9.5440000000000005</v>
+        <v>11</v>
       </c>
       <c r="E79">
-        <v>8.5440000000000005</v>
+        <v>13</v>
       </c>
       <c r="F79">
-        <v>44.8</v>
+        <v>35</v>
       </c>
       <c r="G79">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H79">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="I79" s="13">
-        <v>1.2999999999999999E-2</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A80" s="6"/>
+      <c r="A80" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D80">
+        <v>9.5440000000000005</v>
+      </c>
+      <c r="E80">
+        <v>8.5440000000000005</v>
+      </c>
+      <c r="F80">
+        <v>44.8</v>
+      </c>
+      <c r="G80">
+        <v>30</v>
+      </c>
+      <c r="H80">
+        <v>10</v>
+      </c>
+      <c r="I80" s="13">
+        <v>1.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A81" s="6"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="32" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -11127,7 +11170,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A1" s="11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -11136,7 +11179,7 @@
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A2" s="11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -11145,7 +11188,7 @@
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A3" s="11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="10"/>
@@ -11154,7 +11197,7 @@
     </row>
     <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A4" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -11163,7 +11206,7 @@
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A5" s="11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -11172,7 +11215,7 @@
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A6" s="11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -11181,7 +11224,7 @@
     </row>
     <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A7" s="11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -11190,7 +11233,7 @@
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A8" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -11199,7 +11242,7 @@
     </row>
     <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A9" s="11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -11208,7 +11251,7 @@
     </row>
     <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A10" s="11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -11217,7 +11260,7 @@
     </row>
     <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A11" s="11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -11226,7 +11269,7 @@
     </row>
     <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A12" s="11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -11235,7 +11278,7 @@
     </row>
     <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A13" s="11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -11244,7 +11287,7 @@
     </row>
     <row r="14" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A14" s="11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -11253,7 +11296,7 @@
     </row>
     <row r="15" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A15" s="11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -11262,7 +11305,7 @@
     </row>
     <row r="16" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A16" s="11" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -11271,7 +11314,7 @@
     </row>
     <row r="17" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
       <c r="A17" s="11" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>

</xml_diff>

<commit_message>
update: re-upload latest CaseSize Format.xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Case Size.xlsx
+++ b/Case Size.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ee11846ce882123f/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="297" documentId="8_{B5CB9DC2-2DBC-48FC-8A4C-3FED4FBFDA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56518CD2-2572-42FA-B83D-418CBBC903D3}"/>
+  <xr:revisionPtr revIDLastSave="303" documentId="8_{B5CB9DC2-2DBC-48FC-8A4C-3FED4FBFDA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5374F466-7400-4845-8231-FFC7EA51121C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{94297B88-8998-40EB-8FA5-F929672964CF}"/>
   </bookViews>
@@ -5737,7 +5737,7 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="134" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="134" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -5751,14 +5751,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
@@ -5782,7 +5780,6 @@
     <xf numFmtId="2" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -9167,7 +9164,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{624BC790-9AE4-4E34-8AB5-C11F6DB95162}">
-  <dimension ref="A1:M81"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="41.453125" bestFit="1" customWidth="1"/>
@@ -9178,17 +9175,15 @@
     <col min="6" max="6" width="14.81640625" customWidth="1"/>
     <col min="7" max="7" width="15.453125" customWidth="1"/>
     <col min="8" max="8" width="11.26953125" customWidth="1"/>
-    <col min="9" max="9" width="10.6328125" style="13" customWidth="1"/>
+    <col min="9" max="9" width="10.6328125" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.6">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.6">
+      <c r="A1" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="I1" s="13"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -9198,30 +9193,30 @@
       <c r="C2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="16" t="s">
+      <c r="I2" s="14" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="7"/>
+      <c r="B3" s="6"/>
       <c r="C3" s="3" t="s">
         <v>18</v>
       </c>
@@ -9240,15 +9235,15 @@
       <c r="H3" s="3">
         <v>20</v>
       </c>
-      <c r="I3" s="15">
+      <c r="I3" s="13">
         <v>0.02</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="7"/>
+      <c r="B4" s="6"/>
       <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
@@ -9267,15 +9262,15 @@
       <c r="H4" s="3">
         <v>27.5</v>
       </c>
-      <c r="I4" s="15">
+      <c r="I4" s="13">
         <v>0.04</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="7"/>
+      <c r="B5" s="6"/>
       <c r="C5" s="3" t="s">
         <v>50</v>
       </c>
@@ -9294,15 +9289,15 @@
       <c r="H5" s="3">
         <v>54</v>
       </c>
-      <c r="I5" s="15">
+      <c r="I5" s="13">
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="7"/>
+      <c r="B6" s="6"/>
       <c r="C6" s="3" t="s">
         <v>11</v>
       </c>
@@ -9321,15 +9316,15 @@
       <c r="H6" s="3">
         <v>54</v>
       </c>
-      <c r="I6" s="15">
+      <c r="I6" s="13">
         <v>0.09</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="7" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="7"/>
+      <c r="B7" s="6"/>
       <c r="C7" s="3" t="s">
         <v>9</v>
       </c>
@@ -9348,15 +9343,15 @@
       <c r="H7" s="3">
         <v>53.5</v>
       </c>
-      <c r="I7" s="15">
+      <c r="I7" s="13">
         <v>0.08</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="7"/>
+      <c r="B8" s="6"/>
       <c r="C8" s="3" t="s">
         <v>18</v>
       </c>
@@ -9375,15 +9370,15 @@
       <c r="H8" s="3">
         <v>44</v>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="13">
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="7" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="7"/>
+      <c r="B9" s="6"/>
       <c r="C9" s="3" t="s">
         <v>51</v>
       </c>
@@ -9402,15 +9397,15 @@
       <c r="H9" s="3">
         <v>44.5</v>
       </c>
-      <c r="I9" s="15">
+      <c r="I9" s="13">
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="7" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="7"/>
+      <c r="B10" s="6"/>
       <c r="C10" s="3" t="s">
         <v>19</v>
       </c>
@@ -9429,15 +9424,15 @@
       <c r="H10" s="3">
         <v>45</v>
       </c>
-      <c r="I10" s="15">
+      <c r="I10" s="13">
         <v>0.1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="7" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B11" s="7"/>
+      <c r="B11" s="6"/>
       <c r="C11" s="3" t="s">
         <v>9</v>
       </c>
@@ -9456,16 +9451,15 @@
       <c r="H11" s="3">
         <v>53.5</v>
       </c>
-      <c r="I11" s="15">
+      <c r="I11" s="13">
         <v>8.0851875000000004E-2</v>
       </c>
-      <c r="J11" s="5"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="7" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="7"/>
+      <c r="B12" s="6"/>
       <c r="C12" s="3" t="s">
         <v>11</v>
       </c>
@@ -9484,16 +9478,15 @@
       <c r="H12" s="3">
         <v>45</v>
       </c>
-      <c r="I12" s="12">
+      <c r="I12" s="10">
         <v>0.06</v>
       </c>
-      <c r="J12" s="5"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="7" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="7"/>
+      <c r="B13" s="6"/>
       <c r="C13" s="3" t="s">
         <v>11</v>
       </c>
@@ -9512,16 +9505,15 @@
       <c r="H13" s="3">
         <v>45</v>
       </c>
-      <c r="I13" s="12" t="s">
+      <c r="I13" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J13" s="5"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="7"/>
+      <c r="B14" s="6"/>
       <c r="C14" s="3" t="s">
         <v>15</v>
       </c>
@@ -9540,16 +9532,15 @@
       <c r="H14" s="3">
         <v>51.2</v>
       </c>
-      <c r="I14" s="15">
+      <c r="I14" s="13">
         <v>9.2851200000000009E-2</v>
       </c>
-      <c r="J14" s="5"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" s="7" t="s">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="7"/>
+      <c r="B15" s="6"/>
       <c r="C15" s="3" t="s">
         <v>15</v>
       </c>
@@ -9568,16 +9559,15 @@
       <c r="H15" s="3">
         <v>51.2</v>
       </c>
-      <c r="I15" s="15">
+      <c r="I15" s="13">
         <v>9.2851200000000009E-2</v>
       </c>
-      <c r="J15" s="5"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="7" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="7"/>
+      <c r="B16" s="6"/>
       <c r="C16" s="3" t="s">
         <v>18</v>
       </c>
@@ -9596,16 +9586,15 @@
       <c r="H16" s="3">
         <v>49.5</v>
       </c>
-      <c r="I16" s="15">
+      <c r="I16" s="13">
         <v>0.06</v>
       </c>
-      <c r="J16" s="5"/>
     </row>
-    <row r="17" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="7" t="s">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A17" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="B17" s="7"/>
+      <c r="B17" s="6"/>
       <c r="C17" s="3" t="s">
         <v>43</v>
       </c>
@@ -9624,15 +9613,15 @@
       <c r="H17" s="3">
         <v>32</v>
       </c>
-      <c r="I17" s="15">
+      <c r="I17" s="13">
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A18" s="7" t="s">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="7"/>
+      <c r="B18" s="6"/>
       <c r="C18" s="3" t="s">
         <v>19</v>
       </c>
@@ -9651,16 +9640,15 @@
       <c r="H18" s="3">
         <v>45.5</v>
       </c>
-      <c r="I18" s="15">
+      <c r="I18" s="13">
         <v>5.5E-2</v>
       </c>
-      <c r="J18" s="5"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A19" s="7" t="s">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="7"/>
+      <c r="B19" s="6"/>
       <c r="C19" s="3" t="s">
         <v>19</v>
       </c>
@@ -9679,16 +9667,15 @@
       <c r="H19" s="3">
         <v>16</v>
       </c>
-      <c r="I19" s="15">
+      <c r="I19" s="13">
         <v>1.1368E-2</v>
       </c>
-      <c r="J19" s="5"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A20" s="7" t="s">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A20" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="7"/>
+      <c r="B20" s="6"/>
       <c r="C20" s="3" t="s">
         <v>18</v>
       </c>
@@ -9707,16 +9694,16 @@
       <c r="H20" s="3">
         <v>45</v>
       </c>
-      <c r="I20" s="15">
+      <c r="I20" s="13">
         <v>0.04</v>
       </c>
       <c r="J20" s="3"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B21" s="6"/>
+      <c r="B21" s="5"/>
       <c r="C21" s="3" t="s">
         <v>23</v>
       </c>
@@ -9735,16 +9722,16 @@
       <c r="H21" s="3">
         <v>32</v>
       </c>
-      <c r="I21" s="15">
+      <c r="I21" s="13">
         <v>3.1088000000000001E-2</v>
       </c>
       <c r="J21" s="3"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="s">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A22" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="6"/>
+      <c r="B22" s="5"/>
       <c r="C22" s="3" t="s">
         <v>25</v>
       </c>
@@ -9763,16 +9750,16 @@
       <c r="H22" s="3">
         <v>28.5</v>
       </c>
-      <c r="I22" s="15">
+      <c r="I22" s="13">
         <v>3.5999999999999997E-2</v>
       </c>
       <c r="J22" s="3"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A23" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="6"/>
+      <c r="B23" s="5"/>
       <c r="C23" s="3" t="s">
         <v>26</v>
       </c>
@@ -9791,16 +9778,16 @@
       <c r="H23" s="3">
         <v>48</v>
       </c>
-      <c r="I23" s="15">
+      <c r="I23" s="13">
         <v>4.3999999999999997E-2</v>
       </c>
       <c r="J23" s="3"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="6"/>
+      <c r="B24" s="5"/>
       <c r="C24" s="3" t="s">
         <v>11</v>
       </c>
@@ -9819,16 +9806,16 @@
       <c r="H24" s="3">
         <v>54</v>
       </c>
-      <c r="I24" s="15">
+      <c r="I24" s="13">
         <v>9.9629999999999996E-2</v>
       </c>
       <c r="J24" s="3"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A25" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="6"/>
+      <c r="B25" s="5"/>
       <c r="C25" s="3" t="s">
         <v>28</v>
       </c>
@@ -9847,16 +9834,16 @@
       <c r="H25" s="3">
         <v>35</v>
       </c>
-      <c r="I25" s="15">
+      <c r="I25" s="13">
         <v>9.9015000000000006E-2</v>
       </c>
       <c r="J25" s="3"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A26" s="6" t="s">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A26" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="6"/>
+      <c r="B26" s="5"/>
       <c r="C26" s="3" t="s">
         <v>19</v>
       </c>
@@ -9875,16 +9862,16 @@
       <c r="H26" s="3">
         <v>49</v>
       </c>
-      <c r="I26" s="15">
+      <c r="I26" s="13">
         <v>6.6640000000000005E-2</v>
       </c>
       <c r="J26" s="3"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A27" s="6" t="s">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A27" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="6"/>
+      <c r="B27" s="5"/>
       <c r="C27" s="3" t="s">
         <v>31</v>
       </c>
@@ -9903,16 +9890,16 @@
       <c r="H27" s="3">
         <v>34.799999999999997</v>
       </c>
-      <c r="I27" s="15">
+      <c r="I27" s="13">
         <v>3.6801E-2</v>
       </c>
       <c r="J27" s="3"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A28" s="6" t="s">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A28" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="6"/>
+      <c r="B28" s="5"/>
       <c r="C28" s="3" t="s">
         <v>15</v>
       </c>
@@ -9931,98 +9918,98 @@
       <c r="H28" s="3">
         <v>51.2</v>
       </c>
-      <c r="I28" s="15">
+      <c r="I28" s="13">
         <v>9.2851200000000009E-2</v>
       </c>
       <c r="J28" s="3"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A29" s="6" t="s">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A29" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="6"/>
-      <c r="C29" s="9" t="s">
+      <c r="B29" s="5"/>
+      <c r="C29" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D29" s="9">
+      <c r="D29" s="7">
         <v>13.5</v>
       </c>
-      <c r="E29" s="9">
+      <c r="E29" s="7">
         <v>12.4</v>
       </c>
-      <c r="F29" s="9">
+      <c r="F29" s="7">
         <v>47.5</v>
       </c>
-      <c r="G29" s="9">
+      <c r="G29" s="7">
         <v>44.3</v>
       </c>
-      <c r="H29" s="9">
+      <c r="H29" s="7">
         <v>32.5</v>
       </c>
-      <c r="I29" s="14">
+      <c r="I29" s="12">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="J29" s="6"/>
-      <c r="K29" s="6"/>
-      <c r="L29" s="6"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A30" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="6"/>
-      <c r="C30" s="9" t="s">
+      <c r="B30" s="5"/>
+      <c r="C30" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="7">
         <v>15.3</v>
       </c>
-      <c r="E30" s="9">
+      <c r="E30" s="7">
         <v>13.95</v>
       </c>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="14"/>
-      <c r="J30" s="6"/>
-      <c r="K30" s="6"/>
-      <c r="L30" s="6"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+      <c r="L30" s="5"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A31" s="6" t="s">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A31" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="9" t="s">
+      <c r="B31" s="5"/>
+      <c r="C31" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D31" s="9">
+      <c r="D31" s="7">
         <v>11</v>
       </c>
-      <c r="E31" s="9">
+      <c r="E31" s="7">
         <v>10</v>
       </c>
-      <c r="F31" s="9">
+      <c r="F31" s="7">
         <v>41.5</v>
       </c>
-      <c r="G31" s="9">
+      <c r="G31" s="7">
         <v>27.5</v>
       </c>
-      <c r="H31" s="9">
+      <c r="H31" s="7">
         <v>21</v>
       </c>
-      <c r="I31" s="14">
+      <c r="I31" s="12">
         <v>2.3966250000000001E-2</v>
       </c>
-      <c r="J31" s="6"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="6"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
+      <c r="L31" s="5"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A32" s="7" t="s">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A32" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B32" s="7"/>
+      <c r="B32" s="6"/>
       <c r="C32" s="3" t="s">
         <v>11</v>
       </c>
@@ -10041,19 +10028,15 @@
       <c r="H32" s="3">
         <v>41</v>
       </c>
-      <c r="I32" s="15">
+      <c r="I32" s="13">
         <v>8.2655999999999993E-2</v>
       </c>
-      <c r="J32" s="18"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="18"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A33" s="7" t="s">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A33" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B33" s="7"/>
+      <c r="B33" s="6"/>
       <c r="C33" s="3" t="s">
         <v>40</v>
       </c>
@@ -10072,19 +10055,15 @@
       <c r="H33" s="3">
         <v>46</v>
       </c>
-      <c r="I33" s="15">
+      <c r="I33" s="13">
         <v>5.2999999999999999E-2</v>
       </c>
-      <c r="J33" s="18"/>
-      <c r="K33" s="18"/>
-      <c r="L33" s="18"/>
-      <c r="M33" s="18"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A34" s="7" t="s">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A34" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B34" s="7"/>
+      <c r="B34" s="6"/>
       <c r="C34" s="3" t="s">
         <v>18</v>
       </c>
@@ -10103,19 +10082,15 @@
       <c r="H34" s="3">
         <v>34.5</v>
       </c>
-      <c r="I34" s="15">
+      <c r="I34" s="13">
         <v>2.7047999999999999E-2</v>
       </c>
-      <c r="J34" s="18"/>
-      <c r="K34" s="18"/>
-      <c r="L34" s="18"/>
-      <c r="M34" s="18"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A35" s="7" t="s">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A35" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B35" s="7"/>
+      <c r="B35" s="6"/>
       <c r="C35" s="3" t="s">
         <v>43</v>
       </c>
@@ -10134,19 +10109,15 @@
       <c r="H35" s="3">
         <v>39</v>
       </c>
-      <c r="I35" s="15">
+      <c r="I35" s="13">
         <v>0.03</v>
       </c>
-      <c r="J35" s="18"/>
-      <c r="K35" s="18"/>
-      <c r="L35" s="18"/>
-      <c r="M35" s="18"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A36" s="7" t="s">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A36" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B36" s="7"/>
+      <c r="B36" s="6"/>
       <c r="C36" s="3" t="s">
         <v>18</v>
       </c>
@@ -10165,19 +10136,15 @@
       <c r="H36" s="3">
         <v>34.799999999999997</v>
       </c>
-      <c r="I36" s="15">
+      <c r="I36" s="13">
         <v>3.6801E-2</v>
       </c>
-      <c r="J36" s="18"/>
-      <c r="K36" s="18"/>
-      <c r="L36" s="18"/>
-      <c r="M36" s="18"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A37" s="7" t="s">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A37" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B37" s="7"/>
+      <c r="B37" s="6"/>
       <c r="C37" s="3" t="s">
         <v>47</v>
       </c>
@@ -10196,19 +10163,15 @@
       <c r="H37" s="3">
         <v>54.7</v>
       </c>
-      <c r="I37" s="15">
+      <c r="I37" s="13">
         <v>9.4207075000000001E-2</v>
       </c>
-      <c r="J37" s="18"/>
-      <c r="K37" s="18"/>
-      <c r="L37" s="18"/>
-      <c r="M37" s="18"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A38" s="7" t="s">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A38" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B38" s="7"/>
+      <c r="B38" s="6"/>
       <c r="C38" s="3" t="s">
         <v>19</v>
       </c>
@@ -10227,45 +10190,20 @@
       <c r="H38" s="3">
         <v>60</v>
       </c>
-      <c r="I38" s="15">
+      <c r="I38" s="13">
         <v>0.104</v>
       </c>
-      <c r="J38" s="18"/>
-      <c r="K38" s="18"/>
-      <c r="L38" s="18"/>
-      <c r="M38" s="18"/>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A39" s="18"/>
-      <c r="B39" s="18"/>
-      <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="18"/>
-      <c r="G39" s="18"/>
-      <c r="H39" s="18"/>
-      <c r="J39" s="18"/>
-      <c r="K39" s="18"/>
-      <c r="L39" s="18"/>
-      <c r="M39" s="18"/>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="C39"/>
     </row>
-    <row r="40" spans="1:13" ht="23" x14ac:dyDescent="0.35">
-      <c r="A40" s="20" t="s">
+    <row r="40" spans="1:10" ht="23" x14ac:dyDescent="0.35">
+      <c r="A40" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="18"/>
-      <c r="G40" s="18"/>
-      <c r="H40" s="18"/>
-      <c r="J40" s="18"/>
-      <c r="K40" s="18"/>
-      <c r="L40" s="18"/>
-      <c r="M40" s="18"/>
+      <c r="C40"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>0</v>
       </c>
@@ -10275,35 +10213,31 @@
       <c r="C41" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D41" s="17" t="s">
+      <c r="D41" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E41" s="17" t="s">
+      <c r="E41" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="F41" s="17" t="s">
+      <c r="F41" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="G41" s="17" t="s">
+      <c r="G41" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H41" s="17" t="s">
+      <c r="H41" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="I41" s="16" t="s">
+      <c r="I41" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="J41" s="18"/>
-      <c r="K41" s="18"/>
-      <c r="L41" s="18"/>
-      <c r="M41" s="18"/>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A42" s="6" t="s">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A42" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B42" s="6"/>
-      <c r="C42" s="9" t="s">
+      <c r="B42" s="5"/>
+      <c r="C42" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D42" s="3"/>
@@ -10317,17 +10251,17 @@
       <c r="H42" s="3">
         <v>60</v>
       </c>
-      <c r="I42" s="15">
+      <c r="I42" s="13">
         <v>0.12093840000000002</v>
       </c>
-      <c r="J42" s="6"/>
+      <c r="J42" s="5"/>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A43" s="6" t="s">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A43" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B43" s="6"/>
-      <c r="C43" s="9" t="s">
+      <c r="B43" s="5"/>
+      <c r="C43" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D43" s="3">
@@ -10345,17 +10279,17 @@
       <c r="H43" s="3">
         <v>70</v>
       </c>
-      <c r="I43" s="15">
+      <c r="I43" s="13">
         <v>0.12705</v>
       </c>
-      <c r="J43" s="6"/>
+      <c r="J43" s="5"/>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A44" s="6" t="s">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A44" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B44" s="6"/>
-      <c r="C44" s="9" t="s">
+      <c r="B44" s="5"/>
+      <c r="C44" s="7" t="s">
         <v>70</v>
       </c>
       <c r="D44" s="3">
@@ -10373,17 +10307,17 @@
       <c r="H44" s="3">
         <v>45</v>
       </c>
-      <c r="I44" s="15">
+      <c r="I44" s="13">
         <v>0.11015999999999999</v>
       </c>
-      <c r="J44" s="6"/>
+      <c r="J44" s="5"/>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A45" s="6" t="s">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A45" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="B45" s="6"/>
-      <c r="C45" s="9"/>
+      <c r="B45" s="5"/>
+      <c r="C45" s="7"/>
       <c r="D45" s="3">
         <v>8</v>
       </c>
@@ -10399,17 +10333,17 @@
       <c r="H45" s="3">
         <v>33</v>
       </c>
-      <c r="I45" s="15">
+      <c r="I45" s="13">
         <v>7.0223999999999995E-2</v>
       </c>
-      <c r="J45" s="6"/>
+      <c r="J45" s="5"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A46" s="6" t="s">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A46" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B46" s="6"/>
-      <c r="C46" s="9" t="s">
+      <c r="B46" s="5"/>
+      <c r="C46" s="7" t="s">
         <v>19</v>
       </c>
       <c r="D46" s="3">
@@ -10427,18 +10361,18 @@
       <c r="H46" s="3">
         <v>55</v>
       </c>
-      <c r="I46" s="15">
+      <c r="I46" s="13">
         <f>(F46*G46*H46)/1000000</f>
         <v>9.3348749999999994E-2</v>
       </c>
-      <c r="J46" s="6"/>
+      <c r="J46" s="5"/>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A47" s="6" t="s">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A47" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B47" s="6"/>
-      <c r="C47" s="9" t="s">
+      <c r="B47" s="5"/>
+      <c r="C47" s="7" t="s">
         <v>31</v>
       </c>
       <c r="D47" s="3">
@@ -10456,18 +10390,18 @@
       <c r="H47" s="3">
         <v>33.5</v>
       </c>
-      <c r="I47" s="15">
+      <c r="I47" s="13">
         <f>(F47*G47*H47)/1000000</f>
         <v>3.3767999999999999E-2</v>
       </c>
-      <c r="J47" s="6"/>
+      <c r="J47" s="5"/>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A48" s="6" t="s">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A48" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B48" s="6"/>
-      <c r="C48" s="9" t="s">
+      <c r="B48" s="5"/>
+      <c r="C48" s="7" t="s">
         <v>70</v>
       </c>
       <c r="D48" s="3">
@@ -10485,18 +10419,18 @@
       <c r="H48" s="3">
         <v>55</v>
       </c>
-      <c r="I48" s="15">
+      <c r="I48" s="13">
         <f>(F48*G48*H48)/1000000</f>
         <v>9.3348749999999994E-2</v>
       </c>
-      <c r="J48" s="6"/>
+      <c r="J48" s="5"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A49" s="6" t="s">
+      <c r="A49" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B49" s="6"/>
-      <c r="C49" s="9" t="s">
+      <c r="B49" s="5"/>
+      <c r="C49" s="7" t="s">
         <v>11</v>
       </c>
       <c r="D49" s="3">
@@ -10514,18 +10448,18 @@
       <c r="H49" s="3">
         <v>45</v>
       </c>
-      <c r="I49" s="15">
+      <c r="I49" s="13">
         <f>(F49*G49*H49)/1000000</f>
         <v>5.9534999999999998E-2</v>
       </c>
-      <c r="J49" s="6"/>
+      <c r="J49" s="5"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B50" s="6"/>
-      <c r="C50" s="9" t="s">
+      <c r="B50" s="5"/>
+      <c r="C50" s="7" t="s">
         <v>11</v>
       </c>
       <c r="D50" s="3">
@@ -10543,18 +10477,18 @@
       <c r="H50" s="3">
         <v>45</v>
       </c>
-      <c r="I50" s="15">
+      <c r="I50" s="13">
         <f t="shared" ref="I50" si="0">(F50*G50*H50)/1000000</f>
         <v>5.9534999999999998E-2</v>
       </c>
-      <c r="J50" s="6"/>
+      <c r="J50" s="5"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A51" s="6" t="s">
+      <c r="A51" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B51" s="6"/>
-      <c r="C51" s="9" t="s">
+      <c r="B51" s="5"/>
+      <c r="C51" s="7" t="s">
         <v>71</v>
       </c>
       <c r="D51" s="3">
@@ -10572,17 +10506,17 @@
       <c r="H51" s="3">
         <v>34.5</v>
       </c>
-      <c r="I51" s="15">
+      <c r="I51" s="13">
         <v>2.7047999999999999E-2</v>
       </c>
-      <c r="J51" s="6"/>
+      <c r="J51" s="5"/>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A52" s="6" t="s">
+      <c r="A52" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B52" s="6"/>
-      <c r="C52" s="9" t="s">
+      <c r="B52" s="5"/>
+      <c r="C52" s="7" t="s">
         <v>72</v>
       </c>
       <c r="D52" s="3">
@@ -10600,17 +10534,17 @@
       <c r="H52" s="3">
         <v>34.799999999999997</v>
       </c>
-      <c r="I52" s="15">
+      <c r="I52" s="13">
         <v>3.6801E-2</v>
       </c>
-      <c r="J52" s="6"/>
+      <c r="J52" s="5"/>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B53" s="6"/>
-      <c r="C53" s="9"/>
+      <c r="B53" s="5"/>
+      <c r="C53" s="7"/>
       <c r="D53" s="3">
         <v>16</v>
       </c>
@@ -10626,17 +10560,17 @@
       <c r="H53" s="3">
         <v>21</v>
       </c>
-      <c r="I53" s="15">
+      <c r="I53" s="13">
         <v>9.3348749999999994E-2</v>
       </c>
-      <c r="J53" s="6"/>
+      <c r="J53" s="5"/>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B54" s="6"/>
-      <c r="C54" s="9" t="s">
+      <c r="B54" s="5"/>
+      <c r="C54" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D54" s="3">
@@ -10654,17 +10588,17 @@
       <c r="H54" s="3">
         <v>14.1</v>
       </c>
-      <c r="I54" s="15">
+      <c r="I54" s="13">
         <v>9.4E-2</v>
       </c>
-      <c r="J54" s="6"/>
+      <c r="J54" s="5"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A55" s="6" t="s">
+      <c r="A55" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B55" s="6"/>
-      <c r="C55" s="9" t="s">
+      <c r="B55" s="5"/>
+      <c r="C55" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D55" s="3">
@@ -10682,17 +10616,17 @@
       <c r="H55" s="3">
         <v>14.1</v>
       </c>
-      <c r="I55" s="15">
+      <c r="I55" s="13">
         <v>9.4E-2</v>
       </c>
-      <c r="J55" s="6"/>
+      <c r="J55" s="5"/>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A56" s="6" t="s">
+      <c r="A56" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B56" s="6"/>
-      <c r="C56" s="9" t="s">
+      <c r="B56" s="5"/>
+      <c r="C56" s="7" t="s">
         <v>51</v>
       </c>
       <c r="D56" s="3">
@@ -10710,18 +10644,18 @@
       <c r="H56" s="3">
         <v>44.5</v>
       </c>
-      <c r="I56" s="15">
+      <c r="I56" s="13">
         <f t="shared" ref="I56:I57" si="1">(F56*G56*H56)/1000000</f>
         <v>7.2090000000000001E-2</v>
       </c>
-      <c r="J56" s="6"/>
+      <c r="J56" s="5"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A57" s="6" t="s">
+      <c r="A57" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B57" s="6"/>
-      <c r="C57" s="9" t="s">
+      <c r="B57" s="5"/>
+      <c r="C57" s="7" t="s">
         <v>73</v>
       </c>
       <c r="D57" s="3">
@@ -10739,18 +10673,18 @@
       <c r="H57" s="3">
         <v>42</v>
       </c>
-      <c r="I57" s="15">
+      <c r="I57" s="13">
         <f t="shared" si="1"/>
         <v>8.2498500000000002E-2</v>
       </c>
-      <c r="J57" s="6"/>
+      <c r="J57" s="5"/>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A58" s="6" t="s">
+      <c r="A58" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B58" s="6"/>
-      <c r="C58" s="9" t="s">
+      <c r="B58" s="5"/>
+      <c r="C58" s="7" t="s">
         <v>70</v>
       </c>
       <c r="D58" s="3">
@@ -10771,11 +10705,11 @@
         <f>2.5*18</f>
         <v>45</v>
       </c>
-      <c r="I58" s="15">
+      <c r="I58" s="13">
         <f>(F58*G58*H58)/1000000</f>
         <v>0.11015999999999999</v>
       </c>
-      <c r="J58" s="6"/>
+      <c r="J58" s="5"/>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D59" s="3"/>
@@ -10783,7 +10717,7 @@
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
       <c r="H59" s="3"/>
-      <c r="I59" s="15"/>
+      <c r="I59" s="13"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D60" s="3"/>
@@ -10791,59 +10725,58 @@
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
       <c r="H60" s="3"/>
-      <c r="I60" s="15"/>
+      <c r="I60" s="13"/>
     </row>
     <row r="61" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="A61" s="19" t="s">
+      <c r="A61" s="16" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="62" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="21" t="s">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A62" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B62" s="22" t="s">
+      <c r="B62" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C62" s="23" t="s">
+      <c r="C62" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D62" s="24" t="s">
+      <c r="D62" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="E62" s="24" t="s">
+      <c r="E62" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="F62" s="24" t="s">
+      <c r="F62" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="G62" s="24" t="s">
+      <c r="G62" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="H62" s="24" t="s">
+      <c r="H62" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="I62" s="25" t="s">
+      <c r="I62" s="22" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:10" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="6" t="s">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A63" s="5" t="s">
         <v>74</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D63" s="8">
+      <c r="D63">
         <v>9.6</v>
       </c>
-      <c r="E63" s="8">
+      <c r="E63">
         <v>8.8000000000000007</v>
       </c>
-      <c r="I63" s="13"/>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A64" s="6" t="s">
+      <c r="A64" s="5" t="s">
         <v>74</v>
       </c>
       <c r="C64" s="3" t="s">
@@ -10856,23 +10789,22 @@
         <v>24</v>
       </c>
     </row>
-    <row r="65" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="6" t="s">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A65" s="5" t="s">
         <v>75</v>
       </c>
       <c r="C65" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D65" s="8">
+      <c r="D65">
         <v>12.55</v>
       </c>
-      <c r="E65" s="8">
+      <c r="E65">
         <v>11.45</v>
       </c>
-      <c r="I65" s="13"/>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A66" s="6" t="s">
+      <c r="A66" s="5" t="s">
         <v>75</v>
       </c>
       <c r="C66" s="3" t="s">
@@ -10886,7 +10818,7 @@
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A67" s="6" t="s">
+      <c r="A67" s="5" t="s">
         <v>76</v>
       </c>
       <c r="C67" s="3" t="s">
@@ -10900,7 +10832,7 @@
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A68" s="6" t="s">
+      <c r="A68" s="5" t="s">
         <v>77</v>
       </c>
       <c r="C68" s="3" t="s">
@@ -10913,8 +10845,8 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="69" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="6" t="s">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A69" s="5" t="s">
         <v>78</v>
       </c>
       <c r="C69" s="3" t="s">
@@ -10926,24 +10858,23 @@
       <c r="E69">
         <v>17.239999999999998</v>
       </c>
-      <c r="I69" s="13"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A70" s="6" t="s">
+      <c r="A70" s="5" t="s">
         <v>78</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D70" s="8">
+      <c r="D70">
         <v>17.600000000000001</v>
       </c>
-      <c r="E70" s="8">
+      <c r="E70">
         <v>16.600000000000001</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A71" s="6" t="s">
+      <c r="A71" s="5" t="s">
         <v>79</v>
       </c>
       <c r="C71" s="3" t="s">
@@ -10957,46 +10888,44 @@
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A72" s="6"/>
+      <c r="A72" s="5"/>
     </row>
-    <row r="73" spans="1:9" s="8" customFormat="1" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="A73" s="19" t="s">
+    <row r="73" spans="1:9" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="A73" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="C73" s="3"/>
-      <c r="I73" s="13"/>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A74" s="21" t="s">
+      <c r="A74" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B74" s="22" t="s">
+      <c r="B74" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C74" s="23" t="s">
+      <c r="C74" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D74" s="24" t="s">
+      <c r="D74" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="E74" s="24" t="s">
+      <c r="E74" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="F74" s="24" t="s">
+      <c r="F74" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="G74" s="24" t="s">
+      <c r="G74" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="H74" s="24" t="s">
+      <c r="H74" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="I74" s="25" t="s">
+      <c r="I74" s="22" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A75" s="6" t="s">
+      <c r="A75" s="5" t="s">
         <v>88</v>
       </c>
       <c r="C75" s="3" t="s">
@@ -11017,12 +10946,12 @@
       <c r="H75">
         <v>30</v>
       </c>
-      <c r="I75" s="13">
+      <c r="I75" s="11">
         <v>2.7E-2</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A76" s="6" t="s">
+      <c r="A76" s="5" t="s">
         <v>30</v>
       </c>
       <c r="C76" s="3" t="s">
@@ -11043,12 +10972,12 @@
       <c r="H76">
         <v>34.799999999999997</v>
       </c>
-      <c r="I76" s="13">
+      <c r="I76" s="11">
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A77" s="6" t="s">
+      <c r="A77" s="5" t="s">
         <v>89</v>
       </c>
       <c r="C77" s="3" t="s">
@@ -11069,12 +10998,12 @@
       <c r="H77">
         <v>27</v>
       </c>
-      <c r="I77" s="13">
+      <c r="I77" s="11">
         <v>2.6244E-2</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A78" s="6" t="s">
+      <c r="A78" s="5" t="s">
         <v>90</v>
       </c>
       <c r="C78" s="3" t="s">
@@ -11095,12 +11024,12 @@
       <c r="H78">
         <v>34.799999999999997</v>
       </c>
-      <c r="I78" s="13">
+      <c r="I78" s="11">
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A79" s="6" t="s">
+      <c r="A79" s="5" t="s">
         <v>42</v>
       </c>
       <c r="C79" s="3" t="s">
@@ -11121,12 +11050,12 @@
       <c r="H79">
         <v>39</v>
       </c>
-      <c r="I79" s="13">
+      <c r="I79" s="11">
         <v>0.03</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A80" s="6" t="s">
+      <c r="A80" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C80" s="3" t="s">
@@ -11147,12 +11076,12 @@
       <c r="H80">
         <v>10</v>
       </c>
-      <c r="I80" s="13">
+      <c r="I80" s="11">
         <v>1.2999999999999999E-2</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A81" s="6"/>
+      <c r="A81" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="32" type="noConversion"/>
@@ -11169,157 +11098,157 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
     </row>
     <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
     </row>
     <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
     </row>
     <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
     </row>
     <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A9" s="11" t="s">
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A10" s="11" t="s">
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
     </row>
-    <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A11" s="11" t="s">
+    <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
     </row>
-    <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A12" s="11" t="s">
+    <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
     </row>
-    <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A13" s="11" t="s">
+    <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
     </row>
-    <row r="14" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A14" s="11" t="s">
+    <row r="14" spans="1:5" ht="16.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
     </row>
-    <row r="15" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A15" s="11" t="s">
+    <row r="15" spans="1:5" ht="16.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
     </row>
-    <row r="16" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A16" s="11" t="s">
+    <row r="16" spans="1:5" ht="16.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
     </row>
-    <row r="17" spans="1:5" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="A17" s="11" t="s">
+    <row r="17" spans="1:5" ht="16.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>